<commit_message>
docs(reports): update 400+ test case Excel, HTML & unified security and automation reports
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Passed_Test_Cases.xlsx
+++ b/automation/reports/Excel/Passed_Test_Cases.xlsx
@@ -3375,7 +3375,7 @@
         <v>9</v>
       </c>
       <c r="E2" s="2">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>10</v>
@@ -3395,7 +3395,7 @@
         <v>9</v>
       </c>
       <c r="E3" s="2">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>10</v>
@@ -3415,7 +3415,7 @@
         <v>9</v>
       </c>
       <c r="E4" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>15</v>
@@ -3435,7 +3435,7 @@
         <v>9</v>
       </c>
       <c r="E5" s="2">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>18</v>
@@ -3455,7 +3455,7 @@
         <v>9</v>
       </c>
       <c r="E6" s="2">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>21</v>
@@ -3475,7 +3475,7 @@
         <v>9</v>
       </c>
       <c r="E7" s="2">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>10</v>
@@ -3495,7 +3495,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="2">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>15</v>
@@ -3515,7 +3515,7 @@
         <v>9</v>
       </c>
       <c r="E9" s="2">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>15</v>
@@ -3535,7 +3535,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="2">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>18</v>
@@ -3555,7 +3555,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="2">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>21</v>
@@ -3575,7 +3575,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>10</v>
@@ -3595,7 +3595,7 @@
         <v>9</v>
       </c>
       <c r="E13" s="2">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>15</v>
@@ -3615,7 +3615,7 @@
         <v>9</v>
       </c>
       <c r="E14" s="2">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>15</v>
@@ -3635,7 +3635,7 @@
         <v>9</v>
       </c>
       <c r="E15" s="2">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>18</v>
@@ -3655,7 +3655,7 @@
         <v>9</v>
       </c>
       <c r="E16" s="2">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>21</v>
@@ -3675,7 +3675,7 @@
         <v>9</v>
       </c>
       <c r="E17" s="2">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>10</v>
@@ -3695,7 +3695,7 @@
         <v>9</v>
       </c>
       <c r="E18" s="2">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>15</v>
@@ -3715,7 +3715,7 @@
         <v>9</v>
       </c>
       <c r="E19" s="2">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>15</v>
@@ -3735,7 +3735,7 @@
         <v>9</v>
       </c>
       <c r="E20" s="2">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>18</v>
@@ -3755,7 +3755,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="2">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>21</v>
@@ -3775,7 +3775,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="2">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>10</v>
@@ -3795,7 +3795,7 @@
         <v>9</v>
       </c>
       <c r="E23" s="2">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>15</v>
@@ -3815,7 +3815,7 @@
         <v>9</v>
       </c>
       <c r="E24" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>15</v>
@@ -3835,7 +3835,7 @@
         <v>9</v>
       </c>
       <c r="E25" s="2">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>18</v>
@@ -3855,7 +3855,7 @@
         <v>9</v>
       </c>
       <c r="E26" s="2">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>21</v>
@@ -3875,7 +3875,7 @@
         <v>9</v>
       </c>
       <c r="E27" s="2">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>10</v>
@@ -3895,7 +3895,7 @@
         <v>9</v>
       </c>
       <c r="E28" s="2">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>15</v>
@@ -3915,7 +3915,7 @@
         <v>9</v>
       </c>
       <c r="E29" s="2">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>15</v>
@@ -3935,7 +3935,7 @@
         <v>9</v>
       </c>
       <c r="E30" s="2">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>18</v>
@@ -3955,7 +3955,7 @@
         <v>9</v>
       </c>
       <c r="E31" s="2">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>21</v>
@@ -3975,7 +3975,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="2">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>10</v>
@@ -3995,7 +3995,7 @@
         <v>9</v>
       </c>
       <c r="E33" s="2">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>15</v>
@@ -4015,7 +4015,7 @@
         <v>9</v>
       </c>
       <c r="E34" s="2">
-        <v>27</v>
+        <v>61</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>15</v>
@@ -4035,7 +4035,7 @@
         <v>9</v>
       </c>
       <c r="E35" s="2">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>18</v>
@@ -4055,7 +4055,7 @@
         <v>9</v>
       </c>
       <c r="E36" s="2">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>21</v>
@@ -4075,7 +4075,7 @@
         <v>9</v>
       </c>
       <c r="E37" s="2">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>10</v>
@@ -4095,7 +4095,7 @@
         <v>9</v>
       </c>
       <c r="E38" s="2">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>15</v>
@@ -4115,7 +4115,7 @@
         <v>9</v>
       </c>
       <c r="E39" s="2">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>15</v>
@@ -4135,7 +4135,7 @@
         <v>9</v>
       </c>
       <c r="E40" s="2">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>18</v>
@@ -4155,7 +4155,7 @@
         <v>9</v>
       </c>
       <c r="E41" s="2">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>21</v>
@@ -4175,7 +4175,7 @@
         <v>9</v>
       </c>
       <c r="E42" s="2">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>10</v>
@@ -4195,7 +4195,7 @@
         <v>9</v>
       </c>
       <c r="E43" s="2">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>15</v>
@@ -4215,7 +4215,7 @@
         <v>9</v>
       </c>
       <c r="E44" s="2">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>15</v>
@@ -4235,7 +4235,7 @@
         <v>9</v>
       </c>
       <c r="E45" s="2">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>18</v>
@@ -4255,7 +4255,7 @@
         <v>9</v>
       </c>
       <c r="E46" s="2">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>21</v>
@@ -4275,7 +4275,7 @@
         <v>9</v>
       </c>
       <c r="E47" s="2">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>10</v>
@@ -4295,7 +4295,7 @@
         <v>9</v>
       </c>
       <c r="E48" s="2">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>15</v>
@@ -4315,7 +4315,7 @@
         <v>9</v>
       </c>
       <c r="E49" s="2">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>15</v>
@@ -4335,7 +4335,7 @@
         <v>9</v>
       </c>
       <c r="E50" s="2">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>18</v>
@@ -4355,7 +4355,7 @@
         <v>9</v>
       </c>
       <c r="E51" s="2">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>21</v>
@@ -4375,7 +4375,7 @@
         <v>9</v>
       </c>
       <c r="E52" s="2">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>10</v>
@@ -4395,7 +4395,7 @@
         <v>9</v>
       </c>
       <c r="E53" s="2">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>15</v>
@@ -4415,7 +4415,7 @@
         <v>9</v>
       </c>
       <c r="E54" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>15</v>
@@ -4435,7 +4435,7 @@
         <v>9</v>
       </c>
       <c r="E55" s="2">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>18</v>
@@ -4455,7 +4455,7 @@
         <v>9</v>
       </c>
       <c r="E56" s="2">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="F56" s="2" t="s">
         <v>21</v>
@@ -4475,7 +4475,7 @@
         <v>9</v>
       </c>
       <c r="E57" s="2">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>10</v>
@@ -4495,7 +4495,7 @@
         <v>9</v>
       </c>
       <c r="E58" s="2">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>15</v>
@@ -4515,7 +4515,7 @@
         <v>9</v>
       </c>
       <c r="E59" s="2">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F59" s="2" t="s">
         <v>15</v>
@@ -4535,7 +4535,7 @@
         <v>9</v>
       </c>
       <c r="E60" s="2">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>18</v>
@@ -4555,7 +4555,7 @@
         <v>9</v>
       </c>
       <c r="E61" s="2">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>21</v>
@@ -4575,7 +4575,7 @@
         <v>9</v>
       </c>
       <c r="E62" s="2">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>10</v>
@@ -4595,7 +4595,7 @@
         <v>9</v>
       </c>
       <c r="E63" s="2">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>15</v>
@@ -4615,7 +4615,7 @@
         <v>9</v>
       </c>
       <c r="E64" s="2">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="F64" s="2" t="s">
         <v>15</v>
@@ -4635,7 +4635,7 @@
         <v>9</v>
       </c>
       <c r="E65" s="2">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>18</v>
@@ -4675,7 +4675,7 @@
         <v>9</v>
       </c>
       <c r="E67" s="2">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="F67" s="2" t="s">
         <v>10</v>
@@ -4695,7 +4695,7 @@
         <v>9</v>
       </c>
       <c r="E68" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F68" s="2" t="s">
         <v>15</v>
@@ -4715,7 +4715,7 @@
         <v>9</v>
       </c>
       <c r="E69" s="2">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>15</v>
@@ -4735,7 +4735,7 @@
         <v>9</v>
       </c>
       <c r="E70" s="2">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>18</v>
@@ -4755,7 +4755,7 @@
         <v>9</v>
       </c>
       <c r="E71" s="2">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>21</v>
@@ -4775,7 +4775,7 @@
         <v>9</v>
       </c>
       <c r="E72" s="2">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>10</v>
@@ -4795,7 +4795,7 @@
         <v>9</v>
       </c>
       <c r="E73" s="2">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>15</v>
@@ -4815,7 +4815,7 @@
         <v>9</v>
       </c>
       <c r="E74" s="2">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="F74" s="2" t="s">
         <v>15</v>
@@ -4835,7 +4835,7 @@
         <v>9</v>
       </c>
       <c r="E75" s="2">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="F75" s="2" t="s">
         <v>18</v>
@@ -4855,7 +4855,7 @@
         <v>9</v>
       </c>
       <c r="E76" s="2">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>21</v>
@@ -4875,7 +4875,7 @@
         <v>9</v>
       </c>
       <c r="E77" s="2">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>10</v>
@@ -4895,7 +4895,7 @@
         <v>9</v>
       </c>
       <c r="E78" s="2">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>15</v>
@@ -4915,7 +4915,7 @@
         <v>9</v>
       </c>
       <c r="E79" s="2">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>15</v>
@@ -4935,7 +4935,7 @@
         <v>9</v>
       </c>
       <c r="E80" s="2">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>18</v>
@@ -4955,7 +4955,7 @@
         <v>9</v>
       </c>
       <c r="E81" s="2">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="F81" s="2" t="s">
         <v>21</v>
@@ -4975,7 +4975,7 @@
         <v>9</v>
       </c>
       <c r="E82" s="2">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>10</v>
@@ -4995,7 +4995,7 @@
         <v>9</v>
       </c>
       <c r="E83" s="2">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>15</v>
@@ -5015,7 +5015,7 @@
         <v>9</v>
       </c>
       <c r="E84" s="2">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>15</v>
@@ -5035,7 +5035,7 @@
         <v>9</v>
       </c>
       <c r="E85" s="2">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>18</v>
@@ -5055,7 +5055,7 @@
         <v>9</v>
       </c>
       <c r="E86" s="2">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>21</v>
@@ -5075,7 +5075,7 @@
         <v>9</v>
       </c>
       <c r="E87" s="2">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="F87" s="2" t="s">
         <v>10</v>
@@ -5095,7 +5095,7 @@
         <v>9</v>
       </c>
       <c r="E88" s="2">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>15</v>
@@ -5115,7 +5115,7 @@
         <v>9</v>
       </c>
       <c r="E89" s="2">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="F89" s="2" t="s">
         <v>15</v>
@@ -5135,7 +5135,7 @@
         <v>9</v>
       </c>
       <c r="E90" s="2">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F90" s="2" t="s">
         <v>18</v>
@@ -5155,7 +5155,7 @@
         <v>9</v>
       </c>
       <c r="E91" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F91" s="2" t="s">
         <v>21</v>
@@ -5175,7 +5175,7 @@
         <v>9</v>
       </c>
       <c r="E92" s="2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>10</v>
@@ -5195,7 +5195,7 @@
         <v>9</v>
       </c>
       <c r="E93" s="2">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F93" s="2" t="s">
         <v>15</v>
@@ -5215,7 +5215,7 @@
         <v>9</v>
       </c>
       <c r="E94" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>15</v>
@@ -5235,7 +5235,7 @@
         <v>9</v>
       </c>
       <c r="E95" s="2">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>18</v>
@@ -5255,7 +5255,7 @@
         <v>9</v>
       </c>
       <c r="E96" s="2">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="F96" s="2" t="s">
         <v>21</v>
@@ -5275,7 +5275,7 @@
         <v>9</v>
       </c>
       <c r="E97" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F97" s="2" t="s">
         <v>10</v>
@@ -5315,7 +5315,7 @@
         <v>9</v>
       </c>
       <c r="E99" s="2">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>15</v>
@@ -5335,7 +5335,7 @@
         <v>9</v>
       </c>
       <c r="E100" s="2">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>18</v>
@@ -5355,7 +5355,7 @@
         <v>9</v>
       </c>
       <c r="E101" s="2">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>21</v>
@@ -5375,7 +5375,7 @@
         <v>9</v>
       </c>
       <c r="E102" s="2">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F102" s="2" t="s">
         <v>10</v>
@@ -5395,7 +5395,7 @@
         <v>9</v>
       </c>
       <c r="E103" s="2">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="F103" s="2" t="s">
         <v>15</v>
@@ -5415,7 +5415,7 @@
         <v>9</v>
       </c>
       <c r="E104" s="2">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="F104" s="2" t="s">
         <v>15</v>
@@ -5435,7 +5435,7 @@
         <v>9</v>
       </c>
       <c r="E105" s="2">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F105" s="2" t="s">
         <v>18</v>
@@ -5455,7 +5455,7 @@
         <v>9</v>
       </c>
       <c r="E106" s="2">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>21</v>
@@ -5475,7 +5475,7 @@
         <v>9</v>
       </c>
       <c r="E107" s="2">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>10</v>
@@ -5495,7 +5495,7 @@
         <v>9</v>
       </c>
       <c r="E108" s="2">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="F108" s="2" t="s">
         <v>15</v>
@@ -5515,7 +5515,7 @@
         <v>9</v>
       </c>
       <c r="E109" s="2">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F109" s="2" t="s">
         <v>15</v>
@@ -5535,7 +5535,7 @@
         <v>9</v>
       </c>
       <c r="E110" s="2">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>18</v>
@@ -5555,7 +5555,7 @@
         <v>9</v>
       </c>
       <c r="E111" s="2">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F111" s="2" t="s">
         <v>21</v>
@@ -5575,7 +5575,7 @@
         <v>9</v>
       </c>
       <c r="E112" s="2">
-        <v>13</v>
+        <v>63</v>
       </c>
       <c r="F112" s="2" t="s">
         <v>10</v>
@@ -5595,7 +5595,7 @@
         <v>9</v>
       </c>
       <c r="E113" s="2">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>15</v>
@@ -5615,7 +5615,7 @@
         <v>9</v>
       </c>
       <c r="E114" s="2">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="F114" s="2" t="s">
         <v>15</v>
@@ -5635,7 +5635,7 @@
         <v>9</v>
       </c>
       <c r="E115" s="2">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="F115" s="2" t="s">
         <v>18</v>
@@ -5655,7 +5655,7 @@
         <v>9</v>
       </c>
       <c r="E116" s="2">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F116" s="2" t="s">
         <v>21</v>
@@ -5675,7 +5675,7 @@
         <v>9</v>
       </c>
       <c r="E117" s="2">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="F117" s="2" t="s">
         <v>10</v>
@@ -5695,7 +5695,7 @@
         <v>9</v>
       </c>
       <c r="E118" s="2">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="F118" s="2" t="s">
         <v>15</v>
@@ -5715,7 +5715,7 @@
         <v>9</v>
       </c>
       <c r="E119" s="2">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="F119" s="2" t="s">
         <v>15</v>
@@ -5735,7 +5735,7 @@
         <v>9</v>
       </c>
       <c r="E120" s="2">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F120" s="2" t="s">
         <v>18</v>
@@ -5755,7 +5755,7 @@
         <v>9</v>
       </c>
       <c r="E121" s="2">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F121" s="2" t="s">
         <v>21</v>
@@ -5775,7 +5775,7 @@
         <v>9</v>
       </c>
       <c r="E122" s="2">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="F122" s="2" t="s">
         <v>10</v>
@@ -5795,7 +5795,7 @@
         <v>9</v>
       </c>
       <c r="E123" s="2">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F123" s="2" t="s">
         <v>15</v>
@@ -5815,7 +5815,7 @@
         <v>9</v>
       </c>
       <c r="E124" s="2">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F124" s="2" t="s">
         <v>15</v>
@@ -5835,7 +5835,7 @@
         <v>9</v>
       </c>
       <c r="E125" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F125" s="2" t="s">
         <v>18</v>
@@ -5855,7 +5855,7 @@
         <v>9</v>
       </c>
       <c r="E126" s="2">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="F126" s="2" t="s">
         <v>21</v>
@@ -5875,7 +5875,7 @@
         <v>9</v>
       </c>
       <c r="E127" s="2">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="F127" s="2" t="s">
         <v>10</v>
@@ -5895,7 +5895,7 @@
         <v>9</v>
       </c>
       <c r="E128" s="2">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F128" s="2" t="s">
         <v>15</v>
@@ -5915,7 +5915,7 @@
         <v>9</v>
       </c>
       <c r="E129" s="2">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F129" s="2" t="s">
         <v>15</v>
@@ -5935,7 +5935,7 @@
         <v>9</v>
       </c>
       <c r="E130" s="2">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="F130" s="2" t="s">
         <v>18</v>
@@ -5955,7 +5955,7 @@
         <v>9</v>
       </c>
       <c r="E131" s="2">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="F131" s="2" t="s">
         <v>21</v>
@@ -5995,7 +5995,7 @@
         <v>9</v>
       </c>
       <c r="E133" s="2">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="F133" s="2" t="s">
         <v>15</v>
@@ -6015,7 +6015,7 @@
         <v>9</v>
       </c>
       <c r="E134" s="2">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="F134" s="2" t="s">
         <v>15</v>
@@ -6035,7 +6035,7 @@
         <v>9</v>
       </c>
       <c r="E135" s="2">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="F135" s="2" t="s">
         <v>18</v>
@@ -6055,7 +6055,7 @@
         <v>9</v>
       </c>
       <c r="E136" s="2">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="F136" s="2" t="s">
         <v>21</v>
@@ -6075,7 +6075,7 @@
         <v>9</v>
       </c>
       <c r="E137" s="2">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="F137" s="2" t="s">
         <v>10</v>
@@ -6095,7 +6095,7 @@
         <v>9</v>
       </c>
       <c r="E138" s="2">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="F138" s="2" t="s">
         <v>15</v>
@@ -6115,7 +6115,7 @@
         <v>9</v>
       </c>
       <c r="E139" s="2">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="F139" s="2" t="s">
         <v>15</v>
@@ -6135,7 +6135,7 @@
         <v>9</v>
       </c>
       <c r="E140" s="2">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="F140" s="2" t="s">
         <v>18</v>
@@ -6155,7 +6155,7 @@
         <v>9</v>
       </c>
       <c r="E141" s="2">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F141" s="2" t="s">
         <v>21</v>
@@ -6175,7 +6175,7 @@
         <v>9</v>
       </c>
       <c r="E142" s="2">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="F142" s="2" t="s">
         <v>10</v>
@@ -6195,7 +6195,7 @@
         <v>9</v>
       </c>
       <c r="E143" s="2">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F143" s="2" t="s">
         <v>15</v>
@@ -6215,7 +6215,7 @@
         <v>9</v>
       </c>
       <c r="E144" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F144" s="2" t="s">
         <v>15</v>
@@ -6235,7 +6235,7 @@
         <v>9</v>
       </c>
       <c r="E145" s="2">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="F145" s="2" t="s">
         <v>18</v>
@@ -6255,7 +6255,7 @@
         <v>9</v>
       </c>
       <c r="E146" s="2">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F146" s="2" t="s">
         <v>21</v>
@@ -6275,7 +6275,7 @@
         <v>9</v>
       </c>
       <c r="E147" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F147" s="2" t="s">
         <v>10</v>
@@ -6295,7 +6295,7 @@
         <v>9</v>
       </c>
       <c r="E148" s="2">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="F148" s="2" t="s">
         <v>15</v>
@@ -6315,7 +6315,7 @@
         <v>9</v>
       </c>
       <c r="E149" s="2">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="F149" s="2" t="s">
         <v>15</v>
@@ -6335,7 +6335,7 @@
         <v>9</v>
       </c>
       <c r="E150" s="2">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="F150" s="2" t="s">
         <v>18</v>
@@ -6355,7 +6355,7 @@
         <v>9</v>
       </c>
       <c r="E151" s="2">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="F151" s="2" t="s">
         <v>21</v>
@@ -6375,7 +6375,7 @@
         <v>9</v>
       </c>
       <c r="E152" s="2">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="F152" s="2" t="s">
         <v>10</v>
@@ -6395,7 +6395,7 @@
         <v>9</v>
       </c>
       <c r="E153" s="2">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="F153" s="2" t="s">
         <v>15</v>
@@ -6415,7 +6415,7 @@
         <v>9</v>
       </c>
       <c r="E154" s="2">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F154" s="2" t="s">
         <v>15</v>
@@ -6435,7 +6435,7 @@
         <v>9</v>
       </c>
       <c r="E155" s="2">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="F155" s="2" t="s">
         <v>18</v>
@@ -6455,7 +6455,7 @@
         <v>9</v>
       </c>
       <c r="E156" s="2">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F156" s="2" t="s">
         <v>21</v>
@@ -6475,7 +6475,7 @@
         <v>9</v>
       </c>
       <c r="E157" s="2">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F157" s="2" t="s">
         <v>10</v>
@@ -6495,7 +6495,7 @@
         <v>9</v>
       </c>
       <c r="E158" s="2">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F158" s="2" t="s">
         <v>15</v>
@@ -6515,7 +6515,7 @@
         <v>9</v>
       </c>
       <c r="E159" s="2">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F159" s="2" t="s">
         <v>15</v>
@@ -6535,7 +6535,7 @@
         <v>9</v>
       </c>
       <c r="E160" s="2">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F160" s="2" t="s">
         <v>18</v>
@@ -6555,7 +6555,7 @@
         <v>9</v>
       </c>
       <c r="E161" s="2">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F161" s="2" t="s">
         <v>21</v>
@@ -6575,7 +6575,7 @@
         <v>9</v>
       </c>
       <c r="E162" s="2">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="F162" s="2" t="s">
         <v>10</v>
@@ -6595,7 +6595,7 @@
         <v>9</v>
       </c>
       <c r="E163" s="2">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="F163" s="2" t="s">
         <v>15</v>
@@ -6615,7 +6615,7 @@
         <v>9</v>
       </c>
       <c r="E164" s="2">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F164" s="2" t="s">
         <v>15</v>
@@ -6635,7 +6635,7 @@
         <v>9</v>
       </c>
       <c r="E165" s="2">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F165" s="2" t="s">
         <v>18</v>
@@ -6655,7 +6655,7 @@
         <v>9</v>
       </c>
       <c r="E166" s="2">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F166" s="2" t="s">
         <v>21</v>
@@ -6675,7 +6675,7 @@
         <v>9</v>
       </c>
       <c r="E167" s="2">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="F167" s="2" t="s">
         <v>10</v>
@@ -6695,7 +6695,7 @@
         <v>9</v>
       </c>
       <c r="E168" s="2">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="F168" s="2" t="s">
         <v>15</v>
@@ -6715,7 +6715,7 @@
         <v>9</v>
       </c>
       <c r="E169" s="2">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F169" s="2" t="s">
         <v>15</v>
@@ -6735,7 +6735,7 @@
         <v>9</v>
       </c>
       <c r="E170" s="2">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="F170" s="2" t="s">
         <v>18</v>
@@ -6755,7 +6755,7 @@
         <v>9</v>
       </c>
       <c r="E171" s="2">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="F171" s="2" t="s">
         <v>21</v>
@@ -6775,7 +6775,7 @@
         <v>9</v>
       </c>
       <c r="E172" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F172" s="2" t="s">
         <v>10</v>
@@ -6795,7 +6795,7 @@
         <v>9</v>
       </c>
       <c r="E173" s="2">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="F173" s="2" t="s">
         <v>15</v>
@@ -6815,7 +6815,7 @@
         <v>9</v>
       </c>
       <c r="E174" s="2">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F174" s="2" t="s">
         <v>15</v>
@@ -6835,7 +6835,7 @@
         <v>9</v>
       </c>
       <c r="E175" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F175" s="2" t="s">
         <v>18</v>
@@ -6855,7 +6855,7 @@
         <v>9</v>
       </c>
       <c r="E176" s="2">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F176" s="2" t="s">
         <v>21</v>
@@ -6875,7 +6875,7 @@
         <v>9</v>
       </c>
       <c r="E177" s="2">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="F177" s="2" t="s">
         <v>10</v>
@@ -6895,7 +6895,7 @@
         <v>9</v>
       </c>
       <c r="E178" s="2">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F178" s="2" t="s">
         <v>15</v>
@@ -6915,7 +6915,7 @@
         <v>9</v>
       </c>
       <c r="E179" s="2">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="F179" s="2" t="s">
         <v>15</v>
@@ -6935,7 +6935,7 @@
         <v>9</v>
       </c>
       <c r="E180" s="2">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="F180" s="2" t="s">
         <v>18</v>
@@ -6955,7 +6955,7 @@
         <v>9</v>
       </c>
       <c r="E181" s="2">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="F181" s="2" t="s">
         <v>21</v>
@@ -6975,7 +6975,7 @@
         <v>9</v>
       </c>
       <c r="E182" s="2">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="F182" s="2" t="s">
         <v>10</v>
@@ -6995,7 +6995,7 @@
         <v>9</v>
       </c>
       <c r="E183" s="2">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F183" s="2" t="s">
         <v>15</v>
@@ -7015,7 +7015,7 @@
         <v>9</v>
       </c>
       <c r="E184" s="2">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="F184" s="2" t="s">
         <v>15</v>
@@ -7035,7 +7035,7 @@
         <v>9</v>
       </c>
       <c r="E185" s="2">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="F185" s="2" t="s">
         <v>18</v>
@@ -7055,7 +7055,7 @@
         <v>9</v>
       </c>
       <c r="E186" s="2">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="F186" s="2" t="s">
         <v>21</v>
@@ -7075,7 +7075,7 @@
         <v>9</v>
       </c>
       <c r="E187" s="2">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="F187" s="2" t="s">
         <v>10</v>
@@ -7095,7 +7095,7 @@
         <v>9</v>
       </c>
       <c r="E188" s="2">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F188" s="2" t="s">
         <v>15</v>
@@ -7115,7 +7115,7 @@
         <v>9</v>
       </c>
       <c r="E189" s="2">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F189" s="2" t="s">
         <v>15</v>
@@ -7135,7 +7135,7 @@
         <v>9</v>
       </c>
       <c r="E190" s="2">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="F190" s="2" t="s">
         <v>18</v>
@@ -7155,7 +7155,7 @@
         <v>9</v>
       </c>
       <c r="E191" s="2">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F191" s="2" t="s">
         <v>21</v>
@@ -7175,7 +7175,7 @@
         <v>9</v>
       </c>
       <c r="E192" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F192" s="2" t="s">
         <v>10</v>
@@ -7195,7 +7195,7 @@
         <v>9</v>
       </c>
       <c r="E193" s="2">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="F193" s="2" t="s">
         <v>15</v>
@@ -7215,7 +7215,7 @@
         <v>9</v>
       </c>
       <c r="E194" s="2">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="F194" s="2" t="s">
         <v>15</v>
@@ -7235,7 +7235,7 @@
         <v>9</v>
       </c>
       <c r="E195" s="2">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F195" s="2" t="s">
         <v>18</v>
@@ -7255,7 +7255,7 @@
         <v>9</v>
       </c>
       <c r="E196" s="2">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="F196" s="2" t="s">
         <v>21</v>
@@ -7275,7 +7275,7 @@
         <v>9</v>
       </c>
       <c r="E197" s="2">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F197" s="2" t="s">
         <v>10</v>
@@ -7295,7 +7295,7 @@
         <v>9</v>
       </c>
       <c r="E198" s="2">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="F198" s="2" t="s">
         <v>15</v>
@@ -7315,7 +7315,7 @@
         <v>9</v>
       </c>
       <c r="E199" s="2">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="F199" s="2" t="s">
         <v>15</v>
@@ -7335,7 +7335,7 @@
         <v>9</v>
       </c>
       <c r="E200" s="2">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="F200" s="2" t="s">
         <v>18</v>
@@ -7355,7 +7355,7 @@
         <v>9</v>
       </c>
       <c r="E201" s="2">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F201" s="2" t="s">
         <v>21</v>
@@ -7375,7 +7375,7 @@
         <v>9</v>
       </c>
       <c r="E202" s="2">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="F202" s="2" t="s">
         <v>10</v>
@@ -7395,7 +7395,7 @@
         <v>9</v>
       </c>
       <c r="E203" s="2">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="F203" s="2" t="s">
         <v>15</v>
@@ -7415,7 +7415,7 @@
         <v>9</v>
       </c>
       <c r="E204" s="2">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="F204" s="2" t="s">
         <v>15</v>
@@ -7435,7 +7435,7 @@
         <v>9</v>
       </c>
       <c r="E205" s="2">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F205" s="2" t="s">
         <v>18</v>
@@ -7455,7 +7455,7 @@
         <v>9</v>
       </c>
       <c r="E206" s="2">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="F206" s="2" t="s">
         <v>21</v>
@@ -7475,7 +7475,7 @@
         <v>9</v>
       </c>
       <c r="E207" s="2">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F207" s="2" t="s">
         <v>10</v>
@@ -7495,7 +7495,7 @@
         <v>9</v>
       </c>
       <c r="E208" s="2">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="F208" s="2" t="s">
         <v>15</v>
@@ -7515,7 +7515,7 @@
         <v>9</v>
       </c>
       <c r="E209" s="2">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="F209" s="2" t="s">
         <v>15</v>
@@ -7535,7 +7535,7 @@
         <v>9</v>
       </c>
       <c r="E210" s="2">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="F210" s="2" t="s">
         <v>18</v>
@@ -7575,7 +7575,7 @@
         <v>9</v>
       </c>
       <c r="E212" s="2">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F212" s="2" t="s">
         <v>10</v>
@@ -7595,7 +7595,7 @@
         <v>9</v>
       </c>
       <c r="E213" s="2">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="F213" s="2" t="s">
         <v>15</v>
@@ -7615,7 +7615,7 @@
         <v>9</v>
       </c>
       <c r="E214" s="2">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="F214" s="2" t="s">
         <v>15</v>
@@ -7635,7 +7635,7 @@
         <v>9</v>
       </c>
       <c r="E215" s="2">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="F215" s="2" t="s">
         <v>18</v>
@@ -7655,7 +7655,7 @@
         <v>9</v>
       </c>
       <c r="E216" s="2">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="F216" s="2" t="s">
         <v>21</v>
@@ -7675,7 +7675,7 @@
         <v>9</v>
       </c>
       <c r="E217" s="2">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="F217" s="2" t="s">
         <v>10</v>
@@ -7695,7 +7695,7 @@
         <v>9</v>
       </c>
       <c r="E218" s="2">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="F218" s="2" t="s">
         <v>15</v>
@@ -7715,7 +7715,7 @@
         <v>9</v>
       </c>
       <c r="E219" s="2">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="F219" s="2" t="s">
         <v>15</v>
@@ -7735,7 +7735,7 @@
         <v>9</v>
       </c>
       <c r="E220" s="2">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F220" s="2" t="s">
         <v>18</v>
@@ -7755,7 +7755,7 @@
         <v>9</v>
       </c>
       <c r="E221" s="2">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F221" s="2" t="s">
         <v>21</v>
@@ -7775,7 +7775,7 @@
         <v>9</v>
       </c>
       <c r="E222" s="2">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="F222" s="2" t="s">
         <v>10</v>
@@ -7795,7 +7795,7 @@
         <v>9</v>
       </c>
       <c r="E223" s="2">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="F223" s="2" t="s">
         <v>15</v>
@@ -7815,7 +7815,7 @@
         <v>9</v>
       </c>
       <c r="E224" s="2">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="F224" s="2" t="s">
         <v>15</v>
@@ -7835,7 +7835,7 @@
         <v>9</v>
       </c>
       <c r="E225" s="2">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="F225" s="2" t="s">
         <v>18</v>
@@ -7855,7 +7855,7 @@
         <v>9</v>
       </c>
       <c r="E226" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F226" s="2" t="s">
         <v>21</v>
@@ -7875,7 +7875,7 @@
         <v>9</v>
       </c>
       <c r="E227" s="2">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="F227" s="2" t="s">
         <v>10</v>
@@ -7895,7 +7895,7 @@
         <v>9</v>
       </c>
       <c r="E228" s="2">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F228" s="2" t="s">
         <v>15</v>
@@ -7915,7 +7915,7 @@
         <v>9</v>
       </c>
       <c r="E229" s="2">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="F229" s="2" t="s">
         <v>15</v>
@@ -7935,7 +7935,7 @@
         <v>9</v>
       </c>
       <c r="E230" s="2">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F230" s="2" t="s">
         <v>18</v>
@@ -7955,7 +7955,7 @@
         <v>9</v>
       </c>
       <c r="E231" s="2">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="F231" s="2" t="s">
         <v>21</v>
@@ -7975,7 +7975,7 @@
         <v>9</v>
       </c>
       <c r="E232" s="2">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="F232" s="2" t="s">
         <v>10</v>
@@ -7995,7 +7995,7 @@
         <v>9</v>
       </c>
       <c r="E233" s="2">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="F233" s="2" t="s">
         <v>15</v>
@@ -8015,7 +8015,7 @@
         <v>9</v>
       </c>
       <c r="E234" s="2">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="F234" s="2" t="s">
         <v>15</v>
@@ -8035,7 +8035,7 @@
         <v>9</v>
       </c>
       <c r="E235" s="2">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="F235" s="2" t="s">
         <v>18</v>
@@ -8055,7 +8055,7 @@
         <v>9</v>
       </c>
       <c r="E236" s="2">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="F236" s="2" t="s">
         <v>21</v>
@@ -8075,7 +8075,7 @@
         <v>9</v>
       </c>
       <c r="E237" s="2">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="F237" s="2" t="s">
         <v>10</v>
@@ -8095,7 +8095,7 @@
         <v>9</v>
       </c>
       <c r="E238" s="2">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F238" s="2" t="s">
         <v>15</v>
@@ -8115,7 +8115,7 @@
         <v>9</v>
       </c>
       <c r="E239" s="2">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="F239" s="2" t="s">
         <v>15</v>
@@ -8135,7 +8135,7 @@
         <v>9</v>
       </c>
       <c r="E240" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F240" s="2" t="s">
         <v>18</v>
@@ -8155,7 +8155,7 @@
         <v>9</v>
       </c>
       <c r="E241" s="2">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="F241" s="2" t="s">
         <v>21</v>
@@ -8175,7 +8175,7 @@
         <v>9</v>
       </c>
       <c r="E242" s="2">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="F242" s="2" t="s">
         <v>10</v>
@@ -8195,7 +8195,7 @@
         <v>9</v>
       </c>
       <c r="E243" s="2">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F243" s="2" t="s">
         <v>15</v>
@@ -8215,7 +8215,7 @@
         <v>9</v>
       </c>
       <c r="E244" s="2">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="F244" s="2" t="s">
         <v>15</v>
@@ -8235,7 +8235,7 @@
         <v>9</v>
       </c>
       <c r="E245" s="2">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="F245" s="2" t="s">
         <v>18</v>
@@ -8255,7 +8255,7 @@
         <v>9</v>
       </c>
       <c r="E246" s="2">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="F246" s="2" t="s">
         <v>21</v>
@@ -8275,7 +8275,7 @@
         <v>9</v>
       </c>
       <c r="E247" s="2">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F247" s="2" t="s">
         <v>10</v>
@@ -8295,7 +8295,7 @@
         <v>9</v>
       </c>
       <c r="E248" s="2">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F248" s="2" t="s">
         <v>15</v>
@@ -8315,7 +8315,7 @@
         <v>9</v>
       </c>
       <c r="E249" s="2">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F249" s="2" t="s">
         <v>15</v>
@@ -8335,7 +8335,7 @@
         <v>9</v>
       </c>
       <c r="E250" s="2">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="F250" s="2" t="s">
         <v>18</v>
@@ -8355,7 +8355,7 @@
         <v>9</v>
       </c>
       <c r="E251" s="2">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="F251" s="2" t="s">
         <v>21</v>
@@ -8375,7 +8375,7 @@
         <v>9</v>
       </c>
       <c r="E252" s="2">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F252" s="2" t="s">
         <v>10</v>
@@ -8395,7 +8395,7 @@
         <v>9</v>
       </c>
       <c r="E253" s="2">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F253" s="2" t="s">
         <v>15</v>
@@ -8415,7 +8415,7 @@
         <v>9</v>
       </c>
       <c r="E254" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F254" s="2" t="s">
         <v>15</v>
@@ -8435,7 +8435,7 @@
         <v>9</v>
       </c>
       <c r="E255" s="2">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F255" s="2" t="s">
         <v>18</v>
@@ -8455,7 +8455,7 @@
         <v>9</v>
       </c>
       <c r="E256" s="2">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="F256" s="2" t="s">
         <v>21</v>
@@ -8475,7 +8475,7 @@
         <v>9</v>
       </c>
       <c r="E257" s="2">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F257" s="2" t="s">
         <v>10</v>
@@ -8495,7 +8495,7 @@
         <v>9</v>
       </c>
       <c r="E258" s="2">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F258" s="2" t="s">
         <v>15</v>
@@ -8515,7 +8515,7 @@
         <v>9</v>
       </c>
       <c r="E259" s="2">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F259" s="2" t="s">
         <v>15</v>
@@ -8535,7 +8535,7 @@
         <v>9</v>
       </c>
       <c r="E260" s="2">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="F260" s="2" t="s">
         <v>18</v>
@@ -8555,7 +8555,7 @@
         <v>9</v>
       </c>
       <c r="E261" s="2">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="F261" s="2" t="s">
         <v>21</v>
@@ -8575,7 +8575,7 @@
         <v>9</v>
       </c>
       <c r="E262" s="2">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F262" s="2" t="s">
         <v>10</v>
@@ -8595,7 +8595,7 @@
         <v>9</v>
       </c>
       <c r="E263" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F263" s="2" t="s">
         <v>15</v>
@@ -8615,7 +8615,7 @@
         <v>9</v>
       </c>
       <c r="E264" s="2">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="F264" s="2" t="s">
         <v>15</v>
@@ -8635,7 +8635,7 @@
         <v>9</v>
       </c>
       <c r="E265" s="2">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="F265" s="2" t="s">
         <v>18</v>
@@ -8655,7 +8655,7 @@
         <v>9</v>
       </c>
       <c r="E266" s="2">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F266" s="2" t="s">
         <v>21</v>
@@ -8675,7 +8675,7 @@
         <v>9</v>
       </c>
       <c r="E267" s="2">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F267" s="2" t="s">
         <v>10</v>
@@ -8695,7 +8695,7 @@
         <v>9</v>
       </c>
       <c r="E268" s="2">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F268" s="2" t="s">
         <v>15</v>
@@ -8715,7 +8715,7 @@
         <v>9</v>
       </c>
       <c r="E269" s="2">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="F269" s="2" t="s">
         <v>15</v>
@@ -8735,7 +8735,7 @@
         <v>9</v>
       </c>
       <c r="E270" s="2">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="F270" s="2" t="s">
         <v>18</v>
@@ -8755,7 +8755,7 @@
         <v>9</v>
       </c>
       <c r="E271" s="2">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="F271" s="2" t="s">
         <v>21</v>
@@ -8775,7 +8775,7 @@
         <v>9</v>
       </c>
       <c r="E272" s="2">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F272" s="2" t="s">
         <v>10</v>
@@ -8795,7 +8795,7 @@
         <v>9</v>
       </c>
       <c r="E273" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F273" s="2" t="s">
         <v>15</v>
@@ -8815,7 +8815,7 @@
         <v>9</v>
       </c>
       <c r="E274" s="2">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F274" s="2" t="s">
         <v>15</v>
@@ -8835,7 +8835,7 @@
         <v>9</v>
       </c>
       <c r="E275" s="2">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F275" s="2" t="s">
         <v>18</v>
@@ -8855,7 +8855,7 @@
         <v>9</v>
       </c>
       <c r="E276" s="2">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F276" s="2" t="s">
         <v>21</v>
@@ -8875,7 +8875,7 @@
         <v>9</v>
       </c>
       <c r="E277" s="2">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="F277" s="2" t="s">
         <v>10</v>
@@ -8895,7 +8895,7 @@
         <v>9</v>
       </c>
       <c r="E278" s="2">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F278" s="2" t="s">
         <v>15</v>
@@ -8915,7 +8915,7 @@
         <v>9</v>
       </c>
       <c r="E279" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="F279" s="2" t="s">
         <v>15</v>
@@ -8935,7 +8935,7 @@
         <v>9</v>
       </c>
       <c r="E280" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F280" s="2" t="s">
         <v>18</v>
@@ -8955,7 +8955,7 @@
         <v>9</v>
       </c>
       <c r="E281" s="2">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F281" s="2" t="s">
         <v>21</v>
@@ -8995,7 +8995,7 @@
         <v>9</v>
       </c>
       <c r="E283" s="2">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F283" s="2" t="s">
         <v>15</v>
@@ -9015,7 +9015,7 @@
         <v>9</v>
       </c>
       <c r="E284" s="2">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F284" s="2" t="s">
         <v>15</v>
@@ -9035,7 +9035,7 @@
         <v>9</v>
       </c>
       <c r="E285" s="2">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F285" s="2" t="s">
         <v>18</v>
@@ -9055,7 +9055,7 @@
         <v>9</v>
       </c>
       <c r="E286" s="2">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="F286" s="2" t="s">
         <v>21</v>
@@ -9075,7 +9075,7 @@
         <v>9</v>
       </c>
       <c r="E287" s="2">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="F287" s="2" t="s">
         <v>10</v>
@@ -9095,7 +9095,7 @@
         <v>9</v>
       </c>
       <c r="E288" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F288" s="2" t="s">
         <v>15</v>
@@ -9115,7 +9115,7 @@
         <v>9</v>
       </c>
       <c r="E289" s="2">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="F289" s="2" t="s">
         <v>15</v>
@@ -9135,7 +9135,7 @@
         <v>9</v>
       </c>
       <c r="E290" s="2">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F290" s="2" t="s">
         <v>18</v>
@@ -9155,7 +9155,7 @@
         <v>9</v>
       </c>
       <c r="E291" s="2">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="F291" s="2" t="s">
         <v>21</v>
@@ -9175,7 +9175,7 @@
         <v>9</v>
       </c>
       <c r="E292" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F292" s="2" t="s">
         <v>10</v>
@@ -9195,7 +9195,7 @@
         <v>9</v>
       </c>
       <c r="E293" s="2">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F293" s="2" t="s">
         <v>15</v>
@@ -9215,7 +9215,7 @@
         <v>9</v>
       </c>
       <c r="E294" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="F294" s="2" t="s">
         <v>15</v>
@@ -9235,7 +9235,7 @@
         <v>9</v>
       </c>
       <c r="E295" s="2">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="F295" s="2" t="s">
         <v>18</v>
@@ -9255,7 +9255,7 @@
         <v>9</v>
       </c>
       <c r="E296" s="2">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="F296" s="2" t="s">
         <v>21</v>
@@ -9275,7 +9275,7 @@
         <v>9</v>
       </c>
       <c r="E297" s="2">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F297" s="2" t="s">
         <v>10</v>
@@ -9295,7 +9295,7 @@
         <v>9</v>
       </c>
       <c r="E298" s="2">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F298" s="2" t="s">
         <v>15</v>
@@ -9315,7 +9315,7 @@
         <v>9</v>
       </c>
       <c r="E299" s="2">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="F299" s="2" t="s">
         <v>15</v>
@@ -9335,7 +9335,7 @@
         <v>9</v>
       </c>
       <c r="E300" s="2">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F300" s="2" t="s">
         <v>18</v>
@@ -9355,7 +9355,7 @@
         <v>9</v>
       </c>
       <c r="E301" s="2">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="F301" s="2" t="s">
         <v>21</v>
@@ -9375,7 +9375,7 @@
         <v>9</v>
       </c>
       <c r="E302" s="2">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="F302" s="2" t="s">
         <v>10</v>
@@ -9395,7 +9395,7 @@
         <v>9</v>
       </c>
       <c r="E303" s="2">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="F303" s="2" t="s">
         <v>15</v>
@@ -9415,7 +9415,7 @@
         <v>9</v>
       </c>
       <c r="E304" s="2">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="F304" s="2" t="s">
         <v>15</v>
@@ -9435,7 +9435,7 @@
         <v>9</v>
       </c>
       <c r="E305" s="2">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="F305" s="2" t="s">
         <v>18</v>
@@ -9455,7 +9455,7 @@
         <v>9</v>
       </c>
       <c r="E306" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F306" s="2" t="s">
         <v>21</v>
@@ -9475,7 +9475,7 @@
         <v>9</v>
       </c>
       <c r="E307" s="2">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F307" s="2" t="s">
         <v>10</v>
@@ -9495,7 +9495,7 @@
         <v>9</v>
       </c>
       <c r="E308" s="2">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F308" s="2" t="s">
         <v>15</v>
@@ -9515,7 +9515,7 @@
         <v>9</v>
       </c>
       <c r="E309" s="2">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F309" s="2" t="s">
         <v>15</v>
@@ -9535,7 +9535,7 @@
         <v>9</v>
       </c>
       <c r="E310" s="2">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F310" s="2" t="s">
         <v>18</v>
@@ -9555,7 +9555,7 @@
         <v>9</v>
       </c>
       <c r="E311" s="2">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F311" s="2" t="s">
         <v>21</v>
@@ -9575,7 +9575,7 @@
         <v>9</v>
       </c>
       <c r="E312" s="2">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="F312" s="2" t="s">
         <v>10</v>
@@ -9595,7 +9595,7 @@
         <v>9</v>
       </c>
       <c r="E313" s="2">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F313" s="2" t="s">
         <v>15</v>
@@ -9615,7 +9615,7 @@
         <v>9</v>
       </c>
       <c r="E314" s="2">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="F314" s="2" t="s">
         <v>15</v>
@@ -9635,7 +9635,7 @@
         <v>9</v>
       </c>
       <c r="E315" s="2">
-        <v>34</v>
+        <v>61</v>
       </c>
       <c r="F315" s="2" t="s">
         <v>18</v>
@@ -9655,7 +9655,7 @@
         <v>9</v>
       </c>
       <c r="E316" s="2">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="F316" s="2" t="s">
         <v>21</v>
@@ -9675,7 +9675,7 @@
         <v>9</v>
       </c>
       <c r="E317" s="2">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="F317" s="2" t="s">
         <v>10</v>
@@ -9695,7 +9695,7 @@
         <v>9</v>
       </c>
       <c r="E318" s="2">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F318" s="2" t="s">
         <v>15</v>
@@ -9715,7 +9715,7 @@
         <v>9</v>
       </c>
       <c r="E319" s="2">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="F319" s="2" t="s">
         <v>15</v>
@@ -9735,7 +9735,7 @@
         <v>9</v>
       </c>
       <c r="E320" s="2">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F320" s="2" t="s">
         <v>18</v>
@@ -9755,7 +9755,7 @@
         <v>9</v>
       </c>
       <c r="E321" s="2">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F321" s="2" t="s">
         <v>21</v>
@@ -9775,7 +9775,7 @@
         <v>9</v>
       </c>
       <c r="E322" s="2">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="F322" s="2" t="s">
         <v>10</v>
@@ -9795,7 +9795,7 @@
         <v>9</v>
       </c>
       <c r="E323" s="2">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="F323" s="2" t="s">
         <v>15</v>
@@ -9815,7 +9815,7 @@
         <v>9</v>
       </c>
       <c r="E324" s="2">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="F324" s="2" t="s">
         <v>15</v>
@@ -9835,7 +9835,7 @@
         <v>9</v>
       </c>
       <c r="E325" s="2">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="F325" s="2" t="s">
         <v>18</v>
@@ -9855,7 +9855,7 @@
         <v>9</v>
       </c>
       <c r="E326" s="2">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F326" s="2" t="s">
         <v>21</v>
@@ -9875,7 +9875,7 @@
         <v>9</v>
       </c>
       <c r="E327" s="2">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F327" s="2" t="s">
         <v>10</v>
@@ -9895,7 +9895,7 @@
         <v>9</v>
       </c>
       <c r="E328" s="2">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="F328" s="2" t="s">
         <v>15</v>
@@ -9915,7 +9915,7 @@
         <v>9</v>
       </c>
       <c r="E329" s="2">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F329" s="2" t="s">
         <v>15</v>
@@ -9935,7 +9935,7 @@
         <v>9</v>
       </c>
       <c r="E330" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F330" s="2" t="s">
         <v>18</v>
@@ -9955,7 +9955,7 @@
         <v>9</v>
       </c>
       <c r="E331" s="2">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="F331" s="2" t="s">
         <v>21</v>
@@ -9975,7 +9975,7 @@
         <v>9</v>
       </c>
       <c r="E332" s="2">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="F332" s="2" t="s">
         <v>10</v>
@@ -9995,7 +9995,7 @@
         <v>9</v>
       </c>
       <c r="E333" s="2">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F333" s="2" t="s">
         <v>15</v>
@@ -10015,7 +10015,7 @@
         <v>9</v>
       </c>
       <c r="E334" s="2">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="F334" s="2" t="s">
         <v>15</v>
@@ -10035,7 +10035,7 @@
         <v>9</v>
       </c>
       <c r="E335" s="2">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F335" s="2" t="s">
         <v>18</v>
@@ -10055,7 +10055,7 @@
         <v>9</v>
       </c>
       <c r="E336" s="2">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="F336" s="2" t="s">
         <v>21</v>
@@ -10075,7 +10075,7 @@
         <v>9</v>
       </c>
       <c r="E337" s="2">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F337" s="2" t="s">
         <v>10</v>
@@ -10095,7 +10095,7 @@
         <v>9</v>
       </c>
       <c r="E338" s="2">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="F338" s="2" t="s">
         <v>15</v>
@@ -10135,7 +10135,7 @@
         <v>9</v>
       </c>
       <c r="E340" s="2">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F340" s="2" t="s">
         <v>18</v>
@@ -10155,7 +10155,7 @@
         <v>9</v>
       </c>
       <c r="E341" s="2">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F341" s="2" t="s">
         <v>21</v>
@@ -10175,7 +10175,7 @@
         <v>9</v>
       </c>
       <c r="E342" s="2">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="F342" s="2" t="s">
         <v>10</v>
@@ -10195,7 +10195,7 @@
         <v>9</v>
       </c>
       <c r="E343" s="2">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="F343" s="2" t="s">
         <v>15</v>
@@ -10215,7 +10215,7 @@
         <v>9</v>
       </c>
       <c r="E344" s="2">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="F344" s="2" t="s">
         <v>15</v>
@@ -10235,7 +10235,7 @@
         <v>9</v>
       </c>
       <c r="E345" s="2">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="F345" s="2" t="s">
         <v>18</v>
@@ -10255,7 +10255,7 @@
         <v>9</v>
       </c>
       <c r="E346" s="2">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F346" s="2" t="s">
         <v>21</v>
@@ -10275,7 +10275,7 @@
         <v>9</v>
       </c>
       <c r="E347" s="2">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="F347" s="2" t="s">
         <v>10</v>
@@ -10295,7 +10295,7 @@
         <v>9</v>
       </c>
       <c r="E348" s="2">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="F348" s="2" t="s">
         <v>15</v>
@@ -10335,7 +10335,7 @@
         <v>9</v>
       </c>
       <c r="E350" s="2">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F350" s="2" t="s">
         <v>18</v>
@@ -10355,7 +10355,7 @@
         <v>9</v>
       </c>
       <c r="E351" s="2">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="F351" s="2" t="s">
         <v>21</v>
@@ -10375,7 +10375,7 @@
         <v>9</v>
       </c>
       <c r="E352" s="2">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F352" s="2" t="s">
         <v>10</v>
@@ -10395,7 +10395,7 @@
         <v>9</v>
       </c>
       <c r="E353" s="2">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="F353" s="2" t="s">
         <v>15</v>
@@ -10415,7 +10415,7 @@
         <v>9</v>
       </c>
       <c r="E354" s="2">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="F354" s="2" t="s">
         <v>15</v>
@@ -10435,7 +10435,7 @@
         <v>9</v>
       </c>
       <c r="E355" s="2">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F355" s="2" t="s">
         <v>18</v>
@@ -10455,7 +10455,7 @@
         <v>9</v>
       </c>
       <c r="E356" s="2">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F356" s="2" t="s">
         <v>21</v>
@@ -10475,7 +10475,7 @@
         <v>9</v>
       </c>
       <c r="E357" s="2">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="F357" s="2" t="s">
         <v>10</v>
@@ -10495,7 +10495,7 @@
         <v>9</v>
       </c>
       <c r="E358" s="2">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="F358" s="2" t="s">
         <v>15</v>
@@ -10515,7 +10515,7 @@
         <v>9</v>
       </c>
       <c r="E359" s="2">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="F359" s="2" t="s">
         <v>15</v>
@@ -10535,7 +10535,7 @@
         <v>9</v>
       </c>
       <c r="E360" s="2">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="F360" s="2" t="s">
         <v>18</v>
@@ -10555,7 +10555,7 @@
         <v>9</v>
       </c>
       <c r="E361" s="2">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F361" s="2" t="s">
         <v>21</v>
@@ -10575,7 +10575,7 @@
         <v>9</v>
       </c>
       <c r="E362" s="2">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F362" s="2" t="s">
         <v>10</v>
@@ -10595,7 +10595,7 @@
         <v>9</v>
       </c>
       <c r="E363" s="2">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="F363" s="2" t="s">
         <v>15</v>
@@ -10615,7 +10615,7 @@
         <v>9</v>
       </c>
       <c r="E364" s="2">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="F364" s="2" t="s">
         <v>15</v>
@@ -10635,7 +10635,7 @@
         <v>9</v>
       </c>
       <c r="E365" s="2">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="F365" s="2" t="s">
         <v>18</v>
@@ -10655,7 +10655,7 @@
         <v>9</v>
       </c>
       <c r="E366" s="2">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F366" s="2" t="s">
         <v>21</v>
@@ -10675,7 +10675,7 @@
         <v>9</v>
       </c>
       <c r="E367" s="2">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="F367" s="2" t="s">
         <v>10</v>
@@ -10695,7 +10695,7 @@
         <v>9</v>
       </c>
       <c r="E368" s="2">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F368" s="2" t="s">
         <v>15</v>
@@ -10715,7 +10715,7 @@
         <v>9</v>
       </c>
       <c r="E369" s="2">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F369" s="2" t="s">
         <v>15</v>
@@ -10735,7 +10735,7 @@
         <v>9</v>
       </c>
       <c r="E370" s="2">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="F370" s="2" t="s">
         <v>18</v>
@@ -10755,7 +10755,7 @@
         <v>9</v>
       </c>
       <c r="E371" s="2">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="F371" s="2" t="s">
         <v>21</v>
@@ -10775,7 +10775,7 @@
         <v>9</v>
       </c>
       <c r="E372" s="2">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="F372" s="2" t="s">
         <v>10</v>
@@ -10795,7 +10795,7 @@
         <v>9</v>
       </c>
       <c r="E373" s="2">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="F373" s="2" t="s">
         <v>15</v>
@@ -10815,7 +10815,7 @@
         <v>9</v>
       </c>
       <c r="E374" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F374" s="2" t="s">
         <v>15</v>
@@ -10835,7 +10835,7 @@
         <v>9</v>
       </c>
       <c r="E375" s="2">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="F375" s="2" t="s">
         <v>18</v>
@@ -10855,7 +10855,7 @@
         <v>9</v>
       </c>
       <c r="E376" s="2">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F376" s="2" t="s">
         <v>21</v>
@@ -10875,7 +10875,7 @@
         <v>9</v>
       </c>
       <c r="E377" s="2">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="F377" s="2" t="s">
         <v>10</v>
@@ -10895,7 +10895,7 @@
         <v>9</v>
       </c>
       <c r="E378" s="2">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="F378" s="2" t="s">
         <v>15</v>
@@ -10915,7 +10915,7 @@
         <v>9</v>
       </c>
       <c r="E379" s="2">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="F379" s="2" t="s">
         <v>15</v>
@@ -10935,7 +10935,7 @@
         <v>9</v>
       </c>
       <c r="E380" s="2">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="F380" s="2" t="s">
         <v>18</v>
@@ -10955,7 +10955,7 @@
         <v>9</v>
       </c>
       <c r="E381" s="2">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F381" s="2" t="s">
         <v>21</v>
@@ -10975,7 +10975,7 @@
         <v>9</v>
       </c>
       <c r="E382" s="2">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="F382" s="2" t="s">
         <v>10</v>
@@ -10995,7 +10995,7 @@
         <v>9</v>
       </c>
       <c r="E383" s="2">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F383" s="2" t="s">
         <v>15</v>
@@ -11015,7 +11015,7 @@
         <v>9</v>
       </c>
       <c r="E384" s="2">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="F384" s="2" t="s">
         <v>15</v>
@@ -11035,7 +11035,7 @@
         <v>9</v>
       </c>
       <c r="E385" s="2">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="F385" s="2" t="s">
         <v>18</v>
@@ -11055,7 +11055,7 @@
         <v>9</v>
       </c>
       <c r="E386" s="2">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="F386" s="2" t="s">
         <v>21</v>
@@ -11075,7 +11075,7 @@
         <v>9</v>
       </c>
       <c r="E387" s="2">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="F387" s="2" t="s">
         <v>10</v>
@@ -11095,7 +11095,7 @@
         <v>9</v>
       </c>
       <c r="E388" s="2">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="F388" s="2" t="s">
         <v>15</v>
@@ -11115,7 +11115,7 @@
         <v>9</v>
       </c>
       <c r="E389" s="2">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="F389" s="2" t="s">
         <v>15</v>
@@ -11135,7 +11135,7 @@
         <v>9</v>
       </c>
       <c r="E390" s="2">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F390" s="2" t="s">
         <v>18</v>
@@ -11155,7 +11155,7 @@
         <v>9</v>
       </c>
       <c r="E391" s="2">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F391" s="2" t="s">
         <v>21</v>
@@ -11175,7 +11175,7 @@
         <v>9</v>
       </c>
       <c r="E392" s="2">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="F392" s="2" t="s">
         <v>10</v>
@@ -11195,7 +11195,7 @@
         <v>9</v>
       </c>
       <c r="E393" s="2">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="F393" s="2" t="s">
         <v>15</v>
@@ -11215,7 +11215,7 @@
         <v>9</v>
       </c>
       <c r="E394" s="2">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="F394" s="2" t="s">
         <v>15</v>
@@ -11235,7 +11235,7 @@
         <v>9</v>
       </c>
       <c r="E395" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F395" s="2" t="s">
         <v>18</v>
@@ -11255,7 +11255,7 @@
         <v>9</v>
       </c>
       <c r="E396" s="2">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="F396" s="2" t="s">
         <v>21</v>
@@ -11275,7 +11275,7 @@
         <v>9</v>
       </c>
       <c r="E397" s="2">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="F397" s="2" t="s">
         <v>10</v>
@@ -11295,7 +11295,7 @@
         <v>9</v>
       </c>
       <c r="E398" s="2">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="F398" s="2" t="s">
         <v>15</v>
@@ -11315,7 +11315,7 @@
         <v>9</v>
       </c>
       <c r="E399" s="2">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F399" s="2" t="s">
         <v>15</v>
@@ -11335,7 +11335,7 @@
         <v>9</v>
       </c>
       <c r="E400" s="2">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="F400" s="2" t="s">
         <v>18</v>
@@ -11355,7 +11355,7 @@
         <v>9</v>
       </c>
       <c r="E401" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F401" s="2" t="s">
         <v>21</v>
@@ -11375,7 +11375,7 @@
         <v>9</v>
       </c>
       <c r="E402" s="2">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="F402" s="2" t="s">
         <v>10</v>
@@ -11395,7 +11395,7 @@
         <v>9</v>
       </c>
       <c r="E403" s="2">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F403" s="2" t="s">
         <v>15</v>
@@ -11415,7 +11415,7 @@
         <v>9</v>
       </c>
       <c r="E404" s="2">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F404" s="2" t="s">
         <v>15</v>
@@ -11435,7 +11435,7 @@
         <v>9</v>
       </c>
       <c r="E405" s="2">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="F405" s="2" t="s">
         <v>18</v>
@@ -11455,7 +11455,7 @@
         <v>9</v>
       </c>
       <c r="E406" s="2">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="F406" s="2" t="s">
         <v>21</v>
@@ -11475,7 +11475,7 @@
         <v>9</v>
       </c>
       <c r="E407" s="2">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="F407" s="2" t="s">
         <v>10</v>
@@ -11495,7 +11495,7 @@
         <v>9</v>
       </c>
       <c r="E408" s="2">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="F408" s="2" t="s">
         <v>15</v>
@@ -11515,7 +11515,7 @@
         <v>9</v>
       </c>
       <c r="E409" s="2">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="F409" s="2" t="s">
         <v>15</v>
@@ -11535,7 +11535,7 @@
         <v>9</v>
       </c>
       <c r="E410" s="2">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="F410" s="2" t="s">
         <v>18</v>
@@ -11555,7 +11555,7 @@
         <v>9</v>
       </c>
       <c r="E411" s="2">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F411" s="2" t="s">
         <v>21</v>
@@ -11575,7 +11575,7 @@
         <v>9</v>
       </c>
       <c r="E412" s="2">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="F412" s="2" t="s">
         <v>10</v>
@@ -11595,7 +11595,7 @@
         <v>9</v>
       </c>
       <c r="E413" s="2">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="F413" s="2" t="s">
         <v>15</v>
@@ -11615,7 +11615,7 @@
         <v>9</v>
       </c>
       <c r="E414" s="2">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="F414" s="2" t="s">
         <v>15</v>
@@ -11635,7 +11635,7 @@
         <v>9</v>
       </c>
       <c r="E415" s="2">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F415" s="2" t="s">
         <v>18</v>
@@ -11655,7 +11655,7 @@
         <v>9</v>
       </c>
       <c r="E416" s="2">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="F416" s="2" t="s">
         <v>21</v>
@@ -11675,7 +11675,7 @@
         <v>9</v>
       </c>
       <c r="E417" s="2">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="F417" s="2" t="s">
         <v>10</v>
@@ -11695,7 +11695,7 @@
         <v>9</v>
       </c>
       <c r="E418" s="2">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F418" s="2" t="s">
         <v>15</v>
@@ -11715,7 +11715,7 @@
         <v>9</v>
       </c>
       <c r="E419" s="2">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="F419" s="2" t="s">
         <v>15</v>
@@ -11735,7 +11735,7 @@
         <v>9</v>
       </c>
       <c r="E420" s="2">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F420" s="2" t="s">
         <v>18</v>
@@ -11775,7 +11775,7 @@
         <v>9</v>
       </c>
       <c r="E422" s="2">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F422" s="2" t="s">
         <v>10</v>
@@ -11795,7 +11795,7 @@
         <v>9</v>
       </c>
       <c r="E423" s="2">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="F423" s="2" t="s">
         <v>15</v>
@@ -11815,7 +11815,7 @@
         <v>9</v>
       </c>
       <c r="E424" s="2">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="F424" s="2" t="s">
         <v>15</v>
@@ -11835,7 +11835,7 @@
         <v>9</v>
       </c>
       <c r="E425" s="2">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F425" s="2" t="s">
         <v>18</v>
@@ -11855,7 +11855,7 @@
         <v>9</v>
       </c>
       <c r="E426" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F426" s="2" t="s">
         <v>21</v>
@@ -11875,7 +11875,7 @@
         <v>9</v>
       </c>
       <c r="E427" s="2">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F427" s="2" t="s">
         <v>10</v>
@@ -11895,7 +11895,7 @@
         <v>9</v>
       </c>
       <c r="E428" s="2">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="F428" s="2" t="s">
         <v>15</v>
@@ -11915,7 +11915,7 @@
         <v>9</v>
       </c>
       <c r="E429" s="2">
-        <v>15</v>
+        <v>47</v>
       </c>
       <c r="F429" s="2" t="s">
         <v>15</v>
@@ -11935,7 +11935,7 @@
         <v>9</v>
       </c>
       <c r="E430" s="2">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="F430" s="2" t="s">
         <v>18</v>
@@ -11955,7 +11955,7 @@
         <v>9</v>
       </c>
       <c r="E431" s="2">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F431" s="2" t="s">
         <v>21</v>
@@ -11975,7 +11975,7 @@
         <v>9</v>
       </c>
       <c r="E432" s="2">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F432" s="2" t="s">
         <v>10</v>
@@ -11995,7 +11995,7 @@
         <v>9</v>
       </c>
       <c r="E433" s="2">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="F433" s="2" t="s">
         <v>15</v>
@@ -12015,7 +12015,7 @@
         <v>9</v>
       </c>
       <c r="E434" s="2">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F434" s="2" t="s">
         <v>15</v>
@@ -12035,7 +12035,7 @@
         <v>9</v>
       </c>
       <c r="E435" s="2">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="F435" s="2" t="s">
         <v>18</v>
@@ -12075,7 +12075,7 @@
         <v>9</v>
       </c>
       <c r="E437" s="2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F437" s="2" t="s">
         <v>10</v>
@@ -12095,7 +12095,7 @@
         <v>9</v>
       </c>
       <c r="E438" s="2">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="F438" s="2" t="s">
         <v>15</v>
@@ -12115,7 +12115,7 @@
         <v>9</v>
       </c>
       <c r="E439" s="2">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="F439" s="2" t="s">
         <v>15</v>
@@ -12135,7 +12135,7 @@
         <v>9</v>
       </c>
       <c r="E440" s="2">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="F440" s="2" t="s">
         <v>18</v>
@@ -12155,7 +12155,7 @@
         <v>9</v>
       </c>
       <c r="E441" s="2">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F441" s="2" t="s">
         <v>21</v>
@@ -12175,7 +12175,7 @@
         <v>9</v>
       </c>
       <c r="E442" s="2">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="F442" s="2" t="s">
         <v>10</v>
@@ -12195,7 +12195,7 @@
         <v>9</v>
       </c>
       <c r="E443" s="2">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F443" s="2" t="s">
         <v>15</v>
@@ -12215,7 +12215,7 @@
         <v>9</v>
       </c>
       <c r="E444" s="2">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="F444" s="2" t="s">
         <v>15</v>
@@ -12235,7 +12235,7 @@
         <v>9</v>
       </c>
       <c r="E445" s="2">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="F445" s="2" t="s">
         <v>18</v>
@@ -12255,7 +12255,7 @@
         <v>9</v>
       </c>
       <c r="E446" s="2">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="F446" s="2" t="s">
         <v>21</v>
@@ -12275,7 +12275,7 @@
         <v>9</v>
       </c>
       <c r="E447" s="2">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="F447" s="2" t="s">
         <v>10</v>
@@ -12295,7 +12295,7 @@
         <v>9</v>
       </c>
       <c r="E448" s="2">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="F448" s="2" t="s">
         <v>15</v>
@@ -12315,7 +12315,7 @@
         <v>9</v>
       </c>
       <c r="E449" s="2">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="F449" s="2" t="s">
         <v>15</v>
@@ -12335,7 +12335,7 @@
         <v>9</v>
       </c>
       <c r="E450" s="2">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F450" s="2" t="s">
         <v>18</v>
@@ -12355,7 +12355,7 @@
         <v>9</v>
       </c>
       <c r="E451" s="2">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="F451" s="2" t="s">
         <v>21</v>
@@ -12375,7 +12375,7 @@
         <v>9</v>
       </c>
       <c r="E452" s="2">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F452" s="2" t="s">
         <v>10</v>
@@ -12395,7 +12395,7 @@
         <v>9</v>
       </c>
       <c r="E453" s="2">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="F453" s="2" t="s">
         <v>15</v>
@@ -12415,7 +12415,7 @@
         <v>9</v>
       </c>
       <c r="E454" s="2">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="F454" s="2" t="s">
         <v>15</v>
@@ -12435,7 +12435,7 @@
         <v>9</v>
       </c>
       <c r="E455" s="2">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="F455" s="2" t="s">
         <v>18</v>
@@ -12455,7 +12455,7 @@
         <v>9</v>
       </c>
       <c r="E456" s="2">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F456" s="2" t="s">
         <v>21</v>
@@ -12475,7 +12475,7 @@
         <v>9</v>
       </c>
       <c r="E457" s="2">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F457" s="2" t="s">
         <v>10</v>
@@ -12495,7 +12495,7 @@
         <v>9</v>
       </c>
       <c r="E458" s="2">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F458" s="2" t="s">
         <v>15</v>
@@ -12515,7 +12515,7 @@
         <v>9</v>
       </c>
       <c r="E459" s="2">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="F459" s="2" t="s">
         <v>15</v>
@@ -12535,7 +12535,7 @@
         <v>9</v>
       </c>
       <c r="E460" s="2">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F460" s="2" t="s">
         <v>18</v>
@@ -12555,7 +12555,7 @@
         <v>9</v>
       </c>
       <c r="E461" s="2">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="F461" s="2" t="s">
         <v>21</v>
@@ -12575,7 +12575,7 @@
         <v>9</v>
       </c>
       <c r="E462" s="2">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="F462" s="2" t="s">
         <v>10</v>
@@ -12595,7 +12595,7 @@
         <v>9</v>
       </c>
       <c r="E463" s="2">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="F463" s="2" t="s">
         <v>15</v>
@@ -12615,7 +12615,7 @@
         <v>9</v>
       </c>
       <c r="E464" s="2">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="F464" s="2" t="s">
         <v>15</v>
@@ -12635,7 +12635,7 @@
         <v>9</v>
       </c>
       <c r="E465" s="2">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F465" s="2" t="s">
         <v>18</v>
@@ -12655,7 +12655,7 @@
         <v>9</v>
       </c>
       <c r="E466" s="2">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="F466" s="2" t="s">
         <v>21</v>
@@ -12675,7 +12675,7 @@
         <v>9</v>
       </c>
       <c r="E467" s="2">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="F467" s="2" t="s">
         <v>10</v>
@@ -12695,7 +12695,7 @@
         <v>9</v>
       </c>
       <c r="E468" s="2">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="F468" s="2" t="s">
         <v>15</v>
@@ -12715,7 +12715,7 @@
         <v>9</v>
       </c>
       <c r="E469" s="2">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="F469" s="2" t="s">
         <v>15</v>
@@ -12735,7 +12735,7 @@
         <v>9</v>
       </c>
       <c r="E470" s="2">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="F470" s="2" t="s">
         <v>18</v>
@@ -12755,7 +12755,7 @@
         <v>9</v>
       </c>
       <c r="E471" s="2">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F471" s="2" t="s">
         <v>21</v>

</xml_diff>